<commit_message>
Revise 08 Blue Cells after two rounds of independent review
Corrects the ladder export and its provenance after review, adds the pre-fix and
recalculated workbook fixtures the claims rest on, and tightens the README to what the
committed file stores (formulas, no computed results).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lb6mmFA8TwAdhUWTxQ12Aw
</commit_message>
<xml_diff>
--- a/ideas/08-blue-cells/fixtures/recalculated_by_libreoffice.xlsx
+++ b/ideas/08-blue-cells/fixtures/recalculated_by_libreoffice.xlsx
@@ -760,48 +760,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>155880</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>142560</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="3619440"/>
-          <a:ext cx="6428880" cy="3571560"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -2596,6 +2554,5 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>